<commit_message>
Atualizando o arquivo XLSX
</commit_message>
<xml_diff>
--- a/jogos_2024-08-27.xlsx
+++ b/jogos_2024-08-27.xlsx
@@ -762,7 +762,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Indonesia Liga 1</t>
+          <t>Thailand Thai League T1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -772,23 +772,23 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Borneo</t>
+          <t>Port FC</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Bali United</t>
+          <t>Sukhothai</t>
         </is>
       </c>
       <c r="G3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
         <v>2</v>
       </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1</v>
-      </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
@@ -798,83 +798,83 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>1.8</v>
+        <v>1.28</v>
       </c>
       <c r="M3" t="n">
-        <v>3.73</v>
+        <v>5.61</v>
       </c>
       <c r="N3" t="n">
-        <v>3.93</v>
+        <v>7.72</v>
       </c>
       <c r="O3" t="n">
-        <v>2.38</v>
+        <v>1.64</v>
       </c>
       <c r="P3" t="n">
-        <v>2.38</v>
+        <v>2.98</v>
       </c>
       <c r="Q3" t="n">
-        <v>3.75</v>
+        <v>7.33</v>
       </c>
       <c r="R3" t="n">
-        <v>1.29</v>
+        <v>1.2</v>
       </c>
       <c r="S3" t="n">
-        <v>3.3</v>
+        <v>4</v>
       </c>
       <c r="T3" t="n">
-        <v>2.3</v>
+        <v>2.04</v>
       </c>
       <c r="U3" t="n">
-        <v>1.55</v>
+        <v>1.75</v>
       </c>
       <c r="V3" t="n">
         <v>1.01</v>
       </c>
       <c r="W3" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="X3" t="n">
-        <v>4.33</v>
+        <v>6.5</v>
       </c>
       <c r="Y3" t="n">
-        <v>1.57</v>
+        <v>1.32</v>
       </c>
       <c r="Z3" t="n">
-        <v>2.28</v>
+        <v>2.98</v>
       </c>
       <c r="AA3" t="n">
-        <v>2.4</v>
+        <v>1.79</v>
       </c>
       <c r="AB3" t="n">
-        <v>1.5</v>
+        <v>2.03</v>
       </c>
       <c r="AC3" t="n">
-        <v>1.57</v>
+        <v>1.62</v>
       </c>
       <c r="AD3" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>['40', '73']</t>
+          <t>['8', '16', '85', '90+2']</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['88']</t>
         </is>
       </c>
       <c r="AG3" t="n">
-        <v>1.3</v>
+        <v>1.07</v>
       </c>
       <c r="AH3" t="n">
-        <v>1.88</v>
+        <v>2.75</v>
       </c>
       <c r="AI3" t="n">
-        <v>1.53</v>
+        <v>1.25</v>
       </c>
       <c r="AJ3" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="AK3" s="3" t="n">
         <v>45531.375</v>
@@ -891,7 +891,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thailand Thai League T1</t>
+          <t>Indonesia Liga 1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -901,23 +901,23 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Port FC</t>
+          <t>Borneo</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Sukhothai</t>
+          <t>Bali United</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
         <v>1</v>
       </c>
-      <c r="I4" t="n">
-        <v>2</v>
-      </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
@@ -927,83 +927,83 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>1.28</v>
+        <v>1.8</v>
       </c>
       <c r="M4" t="n">
-        <v>5.61</v>
+        <v>3.73</v>
       </c>
       <c r="N4" t="n">
-        <v>7.72</v>
+        <v>3.93</v>
       </c>
       <c r="O4" t="n">
-        <v>1.64</v>
+        <v>2.38</v>
       </c>
       <c r="P4" t="n">
-        <v>2.98</v>
+        <v>2.38</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.33</v>
+        <v>3.75</v>
       </c>
       <c r="R4" t="n">
-        <v>1.2</v>
+        <v>1.29</v>
       </c>
       <c r="S4" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
       <c r="T4" t="n">
-        <v>2.04</v>
+        <v>2.3</v>
       </c>
       <c r="U4" t="n">
-        <v>1.75</v>
+        <v>1.55</v>
       </c>
       <c r="V4" t="n">
         <v>1.01</v>
       </c>
       <c r="W4" t="n">
-        <v>1.1</v>
+        <v>1.18</v>
       </c>
       <c r="X4" t="n">
-        <v>6.5</v>
+        <v>4.33</v>
       </c>
       <c r="Y4" t="n">
-        <v>1.32</v>
+        <v>1.57</v>
       </c>
       <c r="Z4" t="n">
-        <v>2.98</v>
+        <v>2.28</v>
       </c>
       <c r="AA4" t="n">
-        <v>1.79</v>
+        <v>2.4</v>
       </c>
       <c r="AB4" t="n">
-        <v>2.03</v>
+        <v>1.5</v>
       </c>
       <c r="AC4" t="n">
-        <v>1.62</v>
+        <v>1.57</v>
       </c>
       <c r="AD4" t="n">
-        <v>2.2</v>
+        <v>2.25</v>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>['8', '16', '85', '90+2']</t>
+          <t>['40', '73']</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>['88']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="AG4" t="n">
-        <v>1.07</v>
+        <v>1.3</v>
       </c>
       <c r="AH4" t="n">
-        <v>2.75</v>
+        <v>1.88</v>
       </c>
       <c r="AI4" t="n">
-        <v>1.25</v>
+        <v>1.53</v>
       </c>
       <c r="AJ4" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="AK4" s="3" t="n">
         <v>45531.375</v>
@@ -1417,48 +1417,48 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Utsikten</t>
+          <t>Brage</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Örebro</t>
+          <t>Helsingborg</t>
         </is>
       </c>
       <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
         <v>3</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
         <v>2</v>
       </c>
-      <c r="I8" t="n">
-        <v>2</v>
-      </c>
-      <c r="J8" t="n">
-        <v>1</v>
-      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>2.45</v>
+        <v>2.05</v>
       </c>
       <c r="M8" t="n">
         <v>3.4</v>
       </c>
       <c r="N8" t="n">
-        <v>2.45</v>
+        <v>3.1</v>
       </c>
       <c r="O8" t="n">
-        <v>3.1</v>
+        <v>2.88</v>
       </c>
       <c r="P8" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="Q8" t="n">
-        <v>3.2</v>
+        <v>3.75</v>
       </c>
       <c r="R8" t="n">
         <v>1.36</v>
@@ -1467,59 +1467,59 @@
         <v>3</v>
       </c>
       <c r="T8" t="n">
-        <v>2.63</v>
+        <v>2.75</v>
       </c>
       <c r="U8" t="n">
-        <v>1.44</v>
+        <v>1.4</v>
       </c>
       <c r="V8" t="n">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
       <c r="W8" t="n">
-        <v>1.25</v>
+        <v>1.28</v>
       </c>
       <c r="X8" t="n">
-        <v>3.97</v>
+        <v>3.75</v>
       </c>
       <c r="Y8" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="Z8" t="n">
         <v>1.8</v>
       </c>
-      <c r="Z8" t="n">
-        <v>1.9</v>
-      </c>
       <c r="AA8" t="n">
-        <v>2.95</v>
+        <v>3.1</v>
       </c>
       <c r="AB8" t="n">
-        <v>1.41</v>
+        <v>1.36</v>
       </c>
       <c r="AC8" t="n">
-        <v>1.62</v>
+        <v>1.7</v>
       </c>
       <c r="AD8" t="n">
-        <v>2.2</v>
+        <v>2.05</v>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>['33', '40', '59']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>['25', '69']</t>
+          <t>['36', '45', '77']</t>
         </is>
       </c>
       <c r="AG8" t="n">
-        <v>1.46</v>
+        <v>1.38</v>
       </c>
       <c r="AH8" t="n">
-        <v>1.55</v>
+        <v>1.68</v>
       </c>
       <c r="AI8" t="n">
-        <v>1.83</v>
+        <v>1.67</v>
       </c>
       <c r="AJ8" t="n">
-        <v>2.05</v>
+        <v>2.3</v>
       </c>
       <c r="AK8" s="3" t="n">
         <v>45531.58333333334</v>
@@ -1536,7 +1536,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sweden Superettan</t>
+          <t>Norway First Division</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1546,109 +1546,109 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Brage</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Helsingborg</t>
+          <t>Sandnes Ulf</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="M9" t="n">
+        <v>5</v>
+      </c>
+      <c r="N9" t="n">
+        <v>7</v>
+      </c>
+      <c r="O9" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="P9" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>6</v>
+      </c>
+      <c r="R9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="S9" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="T9" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="U9" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="V9" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="W9" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="X9" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="Z9" t="n">
         <v>3</v>
       </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>2</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>complete</t>
-        </is>
-      </c>
-      <c r="L9" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="M9" t="n">
+      <c r="AA9" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>['22']</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AG9" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="AJ9" t="n">
         <v>3.4</v>
-      </c>
-      <c r="N9" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="O9" t="n">
-        <v>2.88</v>
-      </c>
-      <c r="P9" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="R9" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="S9" t="n">
-        <v>3</v>
-      </c>
-      <c r="T9" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="U9" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="V9" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="W9" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="X9" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>1.88</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AA9" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="AB9" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="AD9" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="AE9" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>['36', '45', '77']</t>
-        </is>
-      </c>
-      <c r="AG9" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="AH9" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="AI9" t="n">
-        <v>1.67</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>2.3</v>
       </c>
       <c r="AK9" s="3" t="n">
         <v>45531.58333333334</v>
@@ -1665,7 +1665,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Norway First Division</t>
+          <t>Sweden Superettan</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1675,109 +1675,109 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Kongsvinger</t>
+          <t>Utsikten</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Sandnes Ulf</t>
+          <t>Örebro</t>
         </is>
       </c>
       <c r="G10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" t="n">
         <v>1</v>
       </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>1.3</v>
+        <v>2.45</v>
       </c>
       <c r="M10" t="n">
-        <v>5</v>
+        <v>3.4</v>
       </c>
       <c r="N10" t="n">
-        <v>7</v>
+        <v>2.45</v>
       </c>
       <c r="O10" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="R10" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="S10" t="n">
+        <v>3</v>
+      </c>
+      <c r="T10" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="U10" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="V10" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="W10" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="X10" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="Y10" t="n">
         <v>1.8</v>
       </c>
-      <c r="P10" t="n">
-        <v>2.88</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>6</v>
-      </c>
-      <c r="R10" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="S10" t="n">
-        <v>4.33</v>
-      </c>
-      <c r="T10" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="U10" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="V10" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="W10" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="X10" t="n">
-        <v>6.15</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>1.33</v>
-      </c>
       <c r="Z10" t="n">
-        <v>3</v>
+        <v>1.9</v>
       </c>
       <c r="AA10" t="n">
-        <v>1.97</v>
+        <v>2.95</v>
       </c>
       <c r="AB10" t="n">
-        <v>1.85</v>
+        <v>1.41</v>
       </c>
       <c r="AC10" t="n">
-        <v>1.53</v>
+        <v>1.62</v>
       </c>
       <c r="AD10" t="n">
-        <v>2.38</v>
+        <v>2.2</v>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>['22']</t>
+          <t>['33', '40', '59']</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['25', '69']</t>
         </is>
       </c>
       <c r="AG10" t="n">
-        <v>1.08</v>
+        <v>1.46</v>
       </c>
       <c r="AH10" t="n">
-        <v>3.05</v>
+        <v>1.55</v>
       </c>
       <c r="AI10" t="n">
-        <v>1.3</v>
+        <v>1.83</v>
       </c>
       <c r="AJ10" t="n">
-        <v>3.4</v>
+        <v>2.05</v>
       </c>
       <c r="AK10" s="3" t="n">
         <v>45531.58333333334</v>
@@ -2062,25 +2062,25 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Al Feiha</t>
+          <t>Al Raed</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Al Nassr</t>
+          <t>Al Quadisiya</t>
         </is>
       </c>
       <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
         <v>1</v>
       </c>
-      <c r="H13" t="n">
-        <v>4</v>
-      </c>
       <c r="I13" t="n">
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -2088,83 +2088,83 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>8.23</v>
+        <v>3.41</v>
       </c>
       <c r="M13" t="n">
-        <v>6.32</v>
+        <v>3.13</v>
       </c>
       <c r="N13" t="n">
-        <v>1.21</v>
+        <v>1.97</v>
       </c>
       <c r="O13" t="n">
-        <v>7</v>
+        <v>4.33</v>
       </c>
       <c r="P13" t="n">
-        <v>2.8</v>
+        <v>2.25</v>
       </c>
       <c r="Q13" t="n">
-        <v>1.62</v>
+        <v>2.38</v>
       </c>
       <c r="R13" t="n">
-        <v>1.18</v>
+        <v>1.33</v>
       </c>
       <c r="S13" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="T13" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="U13" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="V13" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="W13" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="X13" t="n">
         <v>4.33</v>
       </c>
-      <c r="T13" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="U13" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="V13" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="W13" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="X13" t="n">
-        <v>7.5</v>
-      </c>
       <c r="Y13" t="n">
-        <v>1.29</v>
+        <v>1.73</v>
       </c>
       <c r="Z13" t="n">
-        <v>3.3</v>
+        <v>2.08</v>
       </c>
       <c r="AA13" t="n">
-        <v>1.8</v>
+        <v>2.55</v>
       </c>
       <c r="AB13" t="n">
-        <v>1.91</v>
+        <v>1.5</v>
       </c>
       <c r="AC13" t="n">
-        <v>1.57</v>
+        <v>1.67</v>
       </c>
       <c r="AD13" t="n">
-        <v>2.38</v>
+        <v>2.1</v>
       </c>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>['86']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>['5', '45+10', '85', '90+5']</t>
+          <t>['79']</t>
         </is>
       </c>
       <c r="AG13" t="n">
-        <v>3.35</v>
+        <v>2.23</v>
       </c>
       <c r="AH13" t="n">
-        <v>1.07</v>
+        <v>1.13</v>
       </c>
       <c r="AI13" t="n">
-        <v>3.2</v>
+        <v>2.63</v>
       </c>
       <c r="AJ13" t="n">
-        <v>1.33</v>
+        <v>1.5</v>
       </c>
       <c r="AK13" s="3" t="n">
         <v>45531.625</v>
@@ -2191,25 +2191,25 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Al Raed</t>
+          <t>Al Feiha</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Al Quadisiya</t>
+          <t>Al Nassr</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -2217,83 +2217,83 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>3.41</v>
+        <v>8.23</v>
       </c>
       <c r="M14" t="n">
-        <v>3.13</v>
+        <v>6.32</v>
       </c>
       <c r="N14" t="n">
-        <v>1.97</v>
+        <v>1.21</v>
       </c>
       <c r="O14" t="n">
+        <v>7</v>
+      </c>
+      <c r="P14" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="S14" t="n">
         <v>4.33</v>
       </c>
-      <c r="P14" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="Q14" t="n">
+      <c r="T14" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="U14" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="V14" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="W14" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="X14" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="AD14" t="n">
         <v>2.38</v>
       </c>
-      <c r="R14" t="n">
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>['86']</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>['5', '45+10', '85', '90+5']</t>
+        </is>
+      </c>
+      <c r="AG14" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="AJ14" t="n">
         <v>1.33</v>
-      </c>
-      <c r="S14" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="T14" t="n">
-        <v>2.63</v>
-      </c>
-      <c r="U14" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="V14" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="W14" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="X14" t="n">
-        <v>4.33</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>2.55</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AC14" t="n">
-        <v>1.67</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="AE14" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AF14" t="inlineStr">
-        <is>
-          <t>['79']</t>
-        </is>
-      </c>
-      <c r="AG14" t="n">
-        <v>2.23</v>
-      </c>
-      <c r="AH14" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="AI14" t="n">
-        <v>2.63</v>
-      </c>
-      <c r="AJ14" t="n">
-        <v>1.5</v>
       </c>
       <c r="AK14" s="3" t="n">
         <v>45531.625</v>
@@ -2320,25 +2320,25 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Salernitana</t>
+          <t>Cremonese</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Sampdoria</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -2346,83 +2346,83 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>2.38</v>
+        <v>2.15</v>
       </c>
       <c r="M15" t="n">
         <v>3.4</v>
       </c>
       <c r="N15" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="O15" t="n">
-        <v>2.98</v>
+        <v>2.74</v>
       </c>
       <c r="P15" t="n">
-        <v>1.97</v>
+        <v>2.17</v>
       </c>
       <c r="Q15" t="n">
-        <v>3.5</v>
+        <v>3.74</v>
       </c>
       <c r="R15" t="n">
-        <v>1.45</v>
+        <v>1.37</v>
       </c>
       <c r="S15" t="n">
-        <v>2.6</v>
+        <v>2.95</v>
       </c>
       <c r="T15" t="n">
-        <v>2.95</v>
+        <v>2.75</v>
       </c>
       <c r="U15" t="n">
-        <v>1.37</v>
+        <v>1.42</v>
       </c>
       <c r="V15" t="n">
-        <v>1.07</v>
+        <v>1.01</v>
       </c>
       <c r="W15" t="n">
-        <v>1.35</v>
+        <v>1.25</v>
       </c>
       <c r="X15" t="n">
-        <v>3.23</v>
+        <v>3.42</v>
       </c>
       <c r="Y15" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="Z15" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="AA15" t="n">
-        <v>3.67</v>
+        <v>3.04</v>
       </c>
       <c r="AB15" t="n">
-        <v>1.27</v>
+        <v>1.31</v>
       </c>
       <c r="AC15" t="n">
-        <v>1.8</v>
+        <v>1.71</v>
       </c>
       <c r="AD15" t="n">
-        <v>1.95</v>
+        <v>2.06</v>
       </c>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>['1', '60', '85']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>['4', '21']</t>
+          <t>['76']</t>
         </is>
       </c>
       <c r="AG15" t="n">
-        <v>1.37</v>
+        <v>1.36</v>
       </c>
       <c r="AH15" t="n">
-        <v>1.58</v>
+        <v>1.68</v>
       </c>
       <c r="AI15" t="n">
-        <v>1.94</v>
+        <v>1.83</v>
       </c>
       <c r="AJ15" t="n">
-        <v>2.19</v>
+        <v>2.27</v>
       </c>
       <c r="AK15" s="3" t="n">
         <v>45531.64583333334</v>
@@ -2449,12 +2449,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Cittadella</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Pisa</t>
+          <t>Modena</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -2464,10 +2464,10 @@
         <v>1</v>
       </c>
       <c r="I16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -2475,83 +2475,83 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="M16" t="n">
-        <v>3.25</v>
+        <v>3.4</v>
       </c>
       <c r="N16" t="n">
-        <v>2.62</v>
+        <v>3</v>
       </c>
       <c r="O16" t="n">
-        <v>3.24</v>
+        <v>2.8</v>
       </c>
       <c r="P16" t="n">
-        <v>2.05</v>
+        <v>2</v>
       </c>
       <c r="Q16" t="n">
-        <v>3.38</v>
+        <v>3.75</v>
       </c>
       <c r="R16" t="n">
-        <v>1.44</v>
+        <v>1.36</v>
       </c>
       <c r="S16" t="n">
-        <v>2.67</v>
+        <v>2.88</v>
       </c>
       <c r="T16" t="n">
-        <v>3.05</v>
+        <v>3</v>
       </c>
       <c r="U16" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="V16" t="n">
-        <v>1.03</v>
+        <v>1.06</v>
       </c>
       <c r="W16" t="n">
         <v>1.33</v>
       </c>
       <c r="X16" t="n">
-        <v>2.93</v>
+        <v>3.25</v>
       </c>
       <c r="Y16" t="n">
-        <v>2.05</v>
+        <v>1.95</v>
       </c>
       <c r="Z16" t="n">
-        <v>1.68</v>
+        <v>1.75</v>
       </c>
       <c r="AA16" t="n">
-        <v>3.64</v>
+        <v>3.8</v>
       </c>
       <c r="AB16" t="n">
-        <v>1.22</v>
+        <v>1.25</v>
       </c>
       <c r="AC16" t="n">
-        <v>1.84</v>
+        <v>1.8</v>
       </c>
       <c r="AD16" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>['25']</t>
+          <t>['59']</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>['8']</t>
+          <t>['90+3']</t>
         </is>
       </c>
       <c r="AG16" t="n">
-        <v>1.47</v>
+        <v>1.37</v>
       </c>
       <c r="AH16" t="n">
-        <v>1.49</v>
+        <v>1.63</v>
       </c>
       <c r="AI16" t="n">
-        <v>2.06</v>
+        <v>1.78</v>
       </c>
       <c r="AJ16" t="n">
-        <v>2.09</v>
+        <v>2.25</v>
       </c>
       <c r="AK16" s="3" t="n">
         <v>45531.64583333334</v>
@@ -2707,12 +2707,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Cittadella</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Modena</t>
+          <t>Pisa</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -2722,10 +2722,10 @@
         <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -2733,83 +2733,83 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="M18" t="n">
-        <v>3.4</v>
+        <v>3.25</v>
       </c>
       <c r="N18" t="n">
-        <v>3</v>
+        <v>2.62</v>
       </c>
       <c r="O18" t="n">
-        <v>2.8</v>
+        <v>3.24</v>
       </c>
       <c r="P18" t="n">
-        <v>2</v>
+        <v>2.05</v>
       </c>
       <c r="Q18" t="n">
-        <v>3.75</v>
+        <v>3.38</v>
       </c>
       <c r="R18" t="n">
-        <v>1.36</v>
+        <v>1.44</v>
       </c>
       <c r="S18" t="n">
-        <v>2.88</v>
+        <v>2.67</v>
       </c>
       <c r="T18" t="n">
-        <v>3</v>
+        <v>3.05</v>
       </c>
       <c r="U18" t="n">
-        <v>1.33</v>
+        <v>1.35</v>
       </c>
       <c r="V18" t="n">
-        <v>1.06</v>
+        <v>1.03</v>
       </c>
       <c r="W18" t="n">
         <v>1.33</v>
       </c>
       <c r="X18" t="n">
-        <v>3.25</v>
+        <v>2.93</v>
       </c>
       <c r="Y18" t="n">
-        <v>1.95</v>
+        <v>2.05</v>
       </c>
       <c r="Z18" t="n">
-        <v>1.75</v>
+        <v>1.68</v>
       </c>
       <c r="AA18" t="n">
-        <v>3.8</v>
+        <v>3.64</v>
       </c>
       <c r="AB18" t="n">
-        <v>1.25</v>
+        <v>1.22</v>
       </c>
       <c r="AC18" t="n">
-        <v>1.8</v>
+        <v>1.84</v>
       </c>
       <c r="AD18" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>['59']</t>
+          <t>['25']</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>['90+3']</t>
+          <t>['8']</t>
         </is>
       </c>
       <c r="AG18" t="n">
-        <v>1.37</v>
+        <v>1.47</v>
       </c>
       <c r="AH18" t="n">
-        <v>1.63</v>
+        <v>1.49</v>
       </c>
       <c r="AI18" t="n">
-        <v>1.78</v>
+        <v>2.06</v>
       </c>
       <c r="AJ18" t="n">
-        <v>2.25</v>
+        <v>2.09</v>
       </c>
       <c r="AK18" s="3" t="n">
         <v>45531.64583333334</v>
@@ -2836,109 +2836,109 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Carrarese</t>
+          <t>Bari 1908</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Südtirol</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
         <v>1</v>
       </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
       <c r="K19" t="inlineStr">
         <is>
           <t>complete</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="M19" t="n">
-        <v>3.25</v>
+        <v>3.3</v>
       </c>
       <c r="N19" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="O19" t="n">
         <v>3.4</v>
       </c>
       <c r="P19" t="n">
-        <v>2.05</v>
+        <v>2.1</v>
       </c>
       <c r="Q19" t="n">
-        <v>3.25</v>
+        <v>3</v>
       </c>
       <c r="R19" t="n">
-        <v>1.44</v>
+        <v>1.42</v>
       </c>
       <c r="S19" t="n">
-        <v>2.63</v>
+        <v>2.7</v>
       </c>
       <c r="T19" t="n">
-        <v>3.25</v>
+        <v>2.91</v>
       </c>
       <c r="U19" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="V19" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="W19" t="n">
         <v>1.33</v>
       </c>
-      <c r="V19" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="W19" t="n">
-        <v>1.35</v>
-      </c>
       <c r="X19" t="n">
-        <v>2.9</v>
+        <v>3.35</v>
       </c>
       <c r="Y19" t="n">
-        <v>2.25</v>
+        <v>1.95</v>
       </c>
       <c r="Z19" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>['90+3']</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>['19']</t>
+        </is>
+      </c>
+      <c r="AG19" t="n">
         <v>1.55</v>
       </c>
-      <c r="AA19" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="AB19" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="AC19" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="AD19" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="AE19" t="inlineStr">
-        <is>
-          <t>['45', '56']</t>
-        </is>
-      </c>
-      <c r="AF19" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="AG19" t="n">
-        <v>1.47</v>
-      </c>
       <c r="AH19" t="n">
-        <v>1.37</v>
+        <v>1.42</v>
       </c>
       <c r="AI19" t="n">
         <v>2.1</v>
       </c>
       <c r="AJ19" t="n">
-        <v>1.91</v>
+        <v>1.88</v>
       </c>
       <c r="AK19" s="3" t="n">
         <v>45531.64583333334</v>
@@ -2965,25 +2965,25 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bari 1908</t>
+          <t>Carrarese</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Südtirol</t>
         </is>
       </c>
       <c r="G20" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
         <v>1</v>
       </c>
-      <c r="H20" t="n">
-        <v>1</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0</v>
-      </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -2991,83 +2991,83 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
       <c r="M20" t="n">
-        <v>3.3</v>
+        <v>3.25</v>
       </c>
       <c r="N20" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="O20" t="n">
         <v>3.4</v>
       </c>
       <c r="P20" t="n">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="Q20" t="n">
-        <v>3</v>
+        <v>3.25</v>
       </c>
       <c r="R20" t="n">
-        <v>1.42</v>
+        <v>1.44</v>
       </c>
       <c r="S20" t="n">
-        <v>2.7</v>
+        <v>2.63</v>
       </c>
       <c r="T20" t="n">
-        <v>2.91</v>
+        <v>3.25</v>
       </c>
       <c r="U20" t="n">
-        <v>1.38</v>
+        <v>1.33</v>
       </c>
       <c r="V20" t="n">
-        <v>1.06</v>
+        <v>1.08</v>
       </c>
       <c r="W20" t="n">
-        <v>1.33</v>
+        <v>1.35</v>
       </c>
       <c r="X20" t="n">
-        <v>3.35</v>
+        <v>2.9</v>
       </c>
       <c r="Y20" t="n">
-        <v>1.95</v>
+        <v>2.25</v>
       </c>
       <c r="Z20" t="n">
-        <v>1.75</v>
+        <v>1.55</v>
       </c>
       <c r="AA20" t="n">
-        <v>3.53</v>
+        <v>3.9</v>
       </c>
       <c r="AB20" t="n">
-        <v>1.26</v>
+        <v>1.2</v>
       </c>
       <c r="AC20" t="n">
-        <v>1.75</v>
+        <v>1.91</v>
       </c>
       <c r="AD20" t="n">
-        <v>1.95</v>
+        <v>1.91</v>
       </c>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>['90+3']</t>
+          <t>['45', '56']</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>['19']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="AG20" t="n">
-        <v>1.55</v>
+        <v>1.47</v>
       </c>
       <c r="AH20" t="n">
-        <v>1.42</v>
+        <v>1.37</v>
       </c>
       <c r="AI20" t="n">
         <v>2.1</v>
       </c>
       <c r="AJ20" t="n">
-        <v>1.88</v>
+        <v>1.91</v>
       </c>
       <c r="AK20" s="3" t="n">
         <v>45531.64583333334</v>
@@ -3094,25 +3094,25 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Cremonese</t>
+          <t>Salernitana</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Sampdoria</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H21" t="n">
+        <v>2</v>
+      </c>
+      <c r="I21" t="n">
         <v>1</v>
       </c>
-      <c r="I21" t="n">
-        <v>0</v>
-      </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -3120,83 +3120,83 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>2.15</v>
+        <v>2.38</v>
       </c>
       <c r="M21" t="n">
         <v>3.4</v>
       </c>
       <c r="N21" t="n">
-        <v>3.1</v>
+        <v>2.8</v>
       </c>
       <c r="O21" t="n">
-        <v>2.74</v>
+        <v>2.98</v>
       </c>
       <c r="P21" t="n">
-        <v>2.17</v>
+        <v>1.97</v>
       </c>
       <c r="Q21" t="n">
-        <v>3.74</v>
+        <v>3.5</v>
       </c>
       <c r="R21" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="S21" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="T21" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="U21" t="n">
         <v>1.37</v>
       </c>
-      <c r="S21" t="n">
-        <v>2.95</v>
-      </c>
-      <c r="T21" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="U21" t="n">
-        <v>1.42</v>
-      </c>
       <c r="V21" t="n">
-        <v>1.01</v>
+        <v>1.07</v>
       </c>
       <c r="W21" t="n">
-        <v>1.25</v>
+        <v>1.35</v>
       </c>
       <c r="X21" t="n">
-        <v>3.42</v>
+        <v>3.23</v>
       </c>
       <c r="Y21" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="AC21" t="n">
         <v>1.8</v>
       </c>
-      <c r="Z21" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>3.04</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>1.31</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>1.71</v>
-      </c>
       <c r="AD21" t="n">
-        <v>2.06</v>
+        <v>1.95</v>
       </c>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['1', '60', '85']</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>['76']</t>
+          <t>['4', '21']</t>
         </is>
       </c>
       <c r="AG21" t="n">
-        <v>1.36</v>
+        <v>1.37</v>
       </c>
       <c r="AH21" t="n">
-        <v>1.68</v>
+        <v>1.58</v>
       </c>
       <c r="AI21" t="n">
-        <v>1.83</v>
+        <v>1.94</v>
       </c>
       <c r="AJ21" t="n">
-        <v>2.27</v>
+        <v>2.19</v>
       </c>
       <c r="AK21" s="3" t="n">
         <v>45531.64583333334</v>
@@ -3213,7 +3213,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Europe UEFA Champions League</t>
+          <t>Portugal Campeonato de Portugal Group D</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -3223,91 +3223,91 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sparta Praha</t>
+          <t>Louletano</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Malmö FF</t>
+          <t>Moncarapachense</t>
         </is>
       </c>
       <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="M22" t="n">
+        <v>3</v>
+      </c>
+      <c r="N22" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="O22" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="P22" t="n">
         <v>2</v>
       </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>complete</t>
-        </is>
-      </c>
-      <c r="L22" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="M22" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="N22" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="O22" t="n">
-        <v>2.49</v>
-      </c>
-      <c r="P22" t="n">
-        <v>2.44</v>
-      </c>
       <c r="Q22" t="n">
-        <v>4.52</v>
+        <v>4</v>
       </c>
       <c r="R22" t="n">
-        <v>1.32</v>
+        <v>1.5</v>
       </c>
       <c r="S22" t="n">
-        <v>3.22</v>
+        <v>2.4</v>
       </c>
       <c r="T22" t="n">
-        <v>2.46</v>
+        <v>3.3</v>
       </c>
       <c r="U22" t="n">
-        <v>1.51</v>
+        <v>1.29</v>
       </c>
       <c r="V22" t="n">
-        <v>1.04</v>
+        <v>1.08</v>
       </c>
       <c r="W22" t="n">
-        <v>1.23</v>
+        <v>1.44</v>
       </c>
       <c r="X22" t="n">
-        <v>4.27</v>
+        <v>2.6</v>
       </c>
       <c r="Y22" t="n">
-        <v>1.7</v>
+        <v>2.28</v>
       </c>
       <c r="Z22" t="n">
-        <v>2.15</v>
+        <v>1.56</v>
       </c>
       <c r="AA22" t="n">
-        <v>2.74</v>
+        <v>4.33</v>
       </c>
       <c r="AB22" t="n">
-        <v>1.46</v>
+        <v>1.18</v>
       </c>
       <c r="AC22" t="n">
-        <v>1.63</v>
+        <v>2</v>
       </c>
       <c r="AD22" t="n">
-        <v>2.22</v>
+        <v>1.73</v>
       </c>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>['80', '83']</t>
+          <t>['46']</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
@@ -3316,16 +3316,16 @@
         </is>
       </c>
       <c r="AG22" t="n">
-        <v>1.22</v>
+        <v>1.4</v>
       </c>
       <c r="AH22" t="n">
-        <v>1.93</v>
+        <v>1.55</v>
       </c>
       <c r="AI22" t="n">
-        <v>1.58</v>
+        <v>1.73</v>
       </c>
       <c r="AJ22" t="n">
-        <v>2.45</v>
+        <v>2.6</v>
       </c>
       <c r="AK22" s="3" t="n">
         <v>45531.66666666666</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Portugal Campeonato de Portugal Group D</t>
+          <t>Europe UEFA Champions League</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3352,16 +3352,16 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Louletano</t>
+          <t>Sparta Praha</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Moncarapachense</t>
+          <t>Malmö FF</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -3378,65 +3378,65 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>2.3</v>
+        <v>1.8</v>
       </c>
       <c r="M23" t="n">
-        <v>3</v>
+        <v>3.75</v>
       </c>
       <c r="N23" t="n">
-        <v>2.9</v>
+        <v>3.7</v>
       </c>
       <c r="O23" t="n">
-        <v>2.88</v>
+        <v>2.49</v>
       </c>
       <c r="P23" t="n">
-        <v>2</v>
+        <v>2.44</v>
       </c>
       <c r="Q23" t="n">
-        <v>4</v>
+        <v>4.52</v>
       </c>
       <c r="R23" t="n">
-        <v>1.5</v>
+        <v>1.32</v>
       </c>
       <c r="S23" t="n">
-        <v>2.4</v>
+        <v>3.22</v>
       </c>
       <c r="T23" t="n">
-        <v>3.3</v>
+        <v>2.46</v>
       </c>
       <c r="U23" t="n">
-        <v>1.29</v>
+        <v>1.51</v>
       </c>
       <c r="V23" t="n">
-        <v>1.08</v>
+        <v>1.04</v>
       </c>
       <c r="W23" t="n">
-        <v>1.44</v>
+        <v>1.23</v>
       </c>
       <c r="X23" t="n">
-        <v>2.6</v>
+        <v>4.27</v>
       </c>
       <c r="Y23" t="n">
-        <v>2.28</v>
+        <v>1.7</v>
       </c>
       <c r="Z23" t="n">
-        <v>1.56</v>
+        <v>2.15</v>
       </c>
       <c r="AA23" t="n">
-        <v>4.33</v>
+        <v>2.74</v>
       </c>
       <c r="AB23" t="n">
-        <v>1.18</v>
+        <v>1.46</v>
       </c>
       <c r="AC23" t="n">
-        <v>2</v>
+        <v>1.63</v>
       </c>
       <c r="AD23" t="n">
-        <v>1.73</v>
+        <v>2.22</v>
       </c>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>['46']</t>
+          <t>['80', '83']</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -3445,16 +3445,16 @@
         </is>
       </c>
       <c r="AG23" t="n">
-        <v>1.4</v>
+        <v>1.22</v>
       </c>
       <c r="AH23" t="n">
-        <v>1.55</v>
+        <v>1.93</v>
       </c>
       <c r="AI23" t="n">
-        <v>1.73</v>
+        <v>1.58</v>
       </c>
       <c r="AJ23" t="n">
-        <v>2.6</v>
+        <v>2.45</v>
       </c>
       <c r="AK23" s="3" t="n">
         <v>45531.66666666666</v>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Chile Primera División</t>
+          <t>Brazil Serie B</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -4384,12 +4384,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Cobreloa</t>
+          <t>Coritiba</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Coquimbo Unido</t>
+          <t>Avaí</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -4410,65 +4410,65 @@
         </is>
       </c>
       <c r="L31" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="M31" t="n">
         <v>2.95</v>
       </c>
-      <c r="M31" t="n">
-        <v>3.15</v>
-      </c>
       <c r="N31" t="n">
-        <v>2.3</v>
+        <v>4</v>
       </c>
       <c r="O31" t="n">
-        <v>3.7</v>
+        <v>2.63</v>
       </c>
       <c r="P31" t="n">
-        <v>2.22</v>
+        <v>1.91</v>
       </c>
       <c r="Q31" t="n">
-        <v>2.94</v>
+        <v>6</v>
       </c>
       <c r="R31" t="n">
-        <v>1.38</v>
+        <v>1.57</v>
       </c>
       <c r="S31" t="n">
-        <v>2.99</v>
+        <v>2.25</v>
       </c>
       <c r="T31" t="n">
-        <v>2.92</v>
+        <v>3.75</v>
       </c>
       <c r="U31" t="n">
-        <v>1.4</v>
+        <v>1.25</v>
       </c>
       <c r="V31" t="n">
-        <v>1.03</v>
+        <v>1.11</v>
       </c>
       <c r="W31" t="n">
-        <v>1.29</v>
+        <v>1.5</v>
       </c>
       <c r="X31" t="n">
-        <v>3.3</v>
+        <v>2.43</v>
       </c>
       <c r="Y31" t="n">
-        <v>1.91</v>
+        <v>2.25</v>
       </c>
       <c r="Z31" t="n">
-        <v>1.81</v>
+        <v>1.58</v>
       </c>
       <c r="AA31" t="n">
-        <v>3.2</v>
+        <v>5.5</v>
       </c>
       <c r="AB31" t="n">
-        <v>1.3</v>
+        <v>1.14</v>
       </c>
       <c r="AC31" t="n">
-        <v>1.76</v>
+        <v>2.63</v>
       </c>
       <c r="AD31" t="n">
-        <v>2.05</v>
+        <v>1.44</v>
       </c>
       <c r="AE31" t="inlineStr">
         <is>
-          <t>['79']</t>
+          <t>['61']</t>
         </is>
       </c>
       <c r="AF31" t="inlineStr">
@@ -4477,16 +4477,16 @@
         </is>
       </c>
       <c r="AG31" t="n">
-        <v>1.62</v>
+        <v>1.18</v>
       </c>
       <c r="AH31" t="n">
-        <v>1.38</v>
+        <v>1.85</v>
       </c>
       <c r="AI31" t="n">
-        <v>2.2</v>
+        <v>1.53</v>
       </c>
       <c r="AJ31" t="n">
-        <v>1.88</v>
+        <v>3.4</v>
       </c>
       <c r="AK31" s="3" t="n">
         <v>45531.89583333334</v>
@@ -4503,7 +4503,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Brazil Serie B</t>
+          <t>Chile Primera División</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4513,25 +4513,25 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Coritiba</t>
+          <t>Deportes Iquique</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Avaí</t>
+          <t>Copiapó</t>
         </is>
       </c>
       <c r="G32" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" t="n">
         <v>1</v>
       </c>
-      <c r="H32" t="n">
-        <v>0</v>
-      </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -4539,83 +4539,83 @@
         </is>
       </c>
       <c r="L32" t="n">
-        <v>2.05</v>
+        <v>1.75</v>
       </c>
       <c r="M32" t="n">
-        <v>2.95</v>
+        <v>3.75</v>
       </c>
       <c r="N32" t="n">
         <v>4</v>
       </c>
       <c r="O32" t="n">
-        <v>2.63</v>
+        <v>2.3</v>
       </c>
       <c r="P32" t="n">
-        <v>1.91</v>
+        <v>2.3</v>
       </c>
       <c r="Q32" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R32" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="S32" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="T32" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="U32" t="n">
         <v>1.57</v>
       </c>
-      <c r="S32" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="T32" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="U32" t="n">
-        <v>1.25</v>
-      </c>
       <c r="V32" t="n">
-        <v>1.11</v>
+        <v>1.03</v>
       </c>
       <c r="W32" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="X32" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="AB32" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="AC32" t="n">
         <v>1.5</v>
       </c>
-      <c r="X32" t="n">
-        <v>2.43</v>
-      </c>
-      <c r="Y32" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="Z32" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="AA32" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="AB32" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="AC32" t="n">
-        <v>2.63</v>
-      </c>
       <c r="AD32" t="n">
-        <v>1.44</v>
+        <v>2.3</v>
       </c>
       <c r="AE32" t="inlineStr">
         <is>
-          <t>['61']</t>
+          <t>['15', '56']</t>
         </is>
       </c>
       <c r="AF32" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['45+6']</t>
         </is>
       </c>
       <c r="AG32" t="n">
-        <v>1.18</v>
+        <v>1.21</v>
       </c>
       <c r="AH32" t="n">
-        <v>1.85</v>
+        <v>1.77</v>
       </c>
       <c r="AI32" t="n">
-        <v>1.53</v>
+        <v>1.57</v>
       </c>
       <c r="AJ32" t="n">
-        <v>3.4</v>
+        <v>2.44</v>
       </c>
       <c r="AK32" s="3" t="n">
         <v>45531.89583333334</v>
@@ -4642,25 +4642,25 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Deportes Iquique</t>
+          <t>Cobreloa</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Copiapó</t>
+          <t>Coquimbo Unido</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -4668,83 +4668,83 @@
         </is>
       </c>
       <c r="L33" t="n">
-        <v>1.75</v>
+        <v>2.95</v>
       </c>
       <c r="M33" t="n">
-        <v>3.75</v>
+        <v>3.15</v>
       </c>
       <c r="N33" t="n">
-        <v>4</v>
+        <v>2.3</v>
       </c>
       <c r="O33" t="n">
-        <v>2.3</v>
+        <v>3.7</v>
       </c>
       <c r="P33" t="n">
-        <v>2.3</v>
+        <v>2.22</v>
       </c>
       <c r="Q33" t="n">
-        <v>4</v>
+        <v>2.94</v>
       </c>
       <c r="R33" t="n">
-        <v>1.28</v>
+        <v>1.38</v>
       </c>
       <c r="S33" t="n">
-        <v>3.3</v>
+        <v>2.99</v>
       </c>
       <c r="T33" t="n">
-        <v>2.25</v>
+        <v>2.92</v>
       </c>
       <c r="U33" t="n">
-        <v>1.57</v>
+        <v>1.4</v>
       </c>
       <c r="V33" t="n">
         <v>1.03</v>
       </c>
       <c r="W33" t="n">
-        <v>1.14</v>
+        <v>1.29</v>
       </c>
       <c r="X33" t="n">
-        <v>4.6</v>
+        <v>3.3</v>
       </c>
       <c r="Y33" t="n">
-        <v>1.56</v>
+        <v>1.91</v>
       </c>
       <c r="Z33" t="n">
-        <v>2.34</v>
+        <v>1.81</v>
       </c>
       <c r="AA33" t="n">
-        <v>2.35</v>
+        <v>3.2</v>
       </c>
       <c r="AB33" t="n">
-        <v>1.53</v>
+        <v>1.3</v>
       </c>
       <c r="AC33" t="n">
-        <v>1.5</v>
+        <v>1.76</v>
       </c>
       <c r="AD33" t="n">
-        <v>2.3</v>
+        <v>2.05</v>
       </c>
       <c r="AE33" t="inlineStr">
         <is>
-          <t>['15', '56']</t>
+          <t>['79']</t>
         </is>
       </c>
       <c r="AF33" t="inlineStr">
         <is>
-          <t>['45+6']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="AG33" t="n">
-        <v>1.21</v>
+        <v>1.62</v>
       </c>
       <c r="AH33" t="n">
-        <v>1.77</v>
+        <v>1.38</v>
       </c>
       <c r="AI33" t="n">
-        <v>1.57</v>
+        <v>2.2</v>
       </c>
       <c r="AJ33" t="n">
-        <v>2.44</v>
+        <v>1.88</v>
       </c>
       <c r="AK33" s="3" t="n">
         <v>45531.89583333334</v>

</xml_diff>